<commit_message>
Phase 17K complete before Phase 17L Cooling Load + ACC Capacity Surface
</commit_message>
<xml_diff>
--- a/Configuration Library/ACC_1.5MW_GASENGINE_CDU/equipment/ACC_2/ACC_2.xlsx
+++ b/Configuration Library/ACC_1.5MW_GASENGINE_CDU/equipment/ACC_2/ACC_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ArielLuoProjectspue-solver\Configuration Library\ACC_1.5MW_GASENGINE_CDU\equipment\ACC_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A540FF50-E48C-4945-8E02-FA19C35A5B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913A62B4-C3D9-421B-8F23-B98172D065E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9228,10 +9228,10 @@
         <v>1</v>
       </c>
       <c r="C80" s="7">
-        <v>1607</v>
+        <v>1616</v>
       </c>
       <c r="D80" s="7">
-        <v>367.4</v>
+        <v>386</v>
       </c>
       <c r="E80" s="7">
         <v>4.375</v>

</xml_diff>